<commit_message>
latest update before change
</commit_message>
<xml_diff>
--- a/stochastic_data.xlsx
+++ b/stochastic_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\OneDrive\Υπολογιστής\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\OneDrive\Έγγραφα\python\Stochastic-optimization-problem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E1EE3AF-3A34-4F02-8D6E-213531E3C566}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{648FBA82-C18B-49C4-A16F-CE66BB235AFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{3BAA5D3A-7CAC-420F-A88F-653F0B126F94}"/>
   </bookViews>
@@ -230,9 +230,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Θέμα του Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Θέμα Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -270,7 +270,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -376,7 +376,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -518,7 +518,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -526,7 +526,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{273B4FD2-3D7D-49D3-8EDD-5CBE7AE5B5C9}">
-  <dimension ref="A1:Z4"/>
+  <dimension ref="A1:Z5"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -617,7 +617,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="2">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="C2" s="2">
         <v>130</v>
@@ -697,7 +697,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C3" s="3">
         <v>170</v>
@@ -777,7 +777,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="C4" s="2">
         <v>150</v>
@@ -850,6 +850,86 @@
       </c>
       <c r="Z4" s="2">
         <v>150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2">
+        <v>230</v>
+      </c>
+      <c r="D5" s="2">
+        <v>210</v>
+      </c>
+      <c r="E5" s="2">
+        <v>180</v>
+      </c>
+      <c r="F5" s="2">
+        <v>220</v>
+      </c>
+      <c r="G5" s="2">
+        <v>300</v>
+      </c>
+      <c r="H5" s="2">
+        <v>150</v>
+      </c>
+      <c r="I5" s="2">
+        <v>260</v>
+      </c>
+      <c r="J5" s="2">
+        <v>190</v>
+      </c>
+      <c r="K5" s="2">
+        <v>110</v>
+      </c>
+      <c r="L5" s="2">
+        <v>240</v>
+      </c>
+      <c r="M5" s="2">
+        <v>200</v>
+      </c>
+      <c r="N5" s="2">
+        <v>290</v>
+      </c>
+      <c r="O5" s="2">
+        <v>140</v>
+      </c>
+      <c r="P5" s="2">
+        <v>250</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>180</v>
+      </c>
+      <c r="R5" s="2">
+        <v>270</v>
+      </c>
+      <c r="S5" s="2">
+        <v>160</v>
+      </c>
+      <c r="T5" s="2">
+        <v>230</v>
+      </c>
+      <c r="U5" s="2">
+        <v>120</v>
+      </c>
+      <c r="V5" s="2">
+        <v>210</v>
+      </c>
+      <c r="W5" s="2">
+        <v>100</v>
+      </c>
+      <c r="X5" s="2">
+        <v>300</v>
+      </c>
+      <c r="Y5" s="2">
+        <v>170</v>
+      </c>
+      <c r="Z5" s="2">
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -941,10 +1021,10 @@
         <v>5</v>
       </c>
       <c r="C2" s="2">
-        <v>320</v>
+        <v>1000</v>
       </c>
       <c r="D2" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" s="2">
         <v>1</v>
@@ -958,10 +1038,10 @@
         <v>5</v>
       </c>
       <c r="C3" s="3">
-        <v>390</v>
+        <v>2000</v>
       </c>
       <c r="D3" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E3" s="3">
         <v>2</v>
@@ -972,13 +1052,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2">
+        <v>2500</v>
+      </c>
+      <c r="D4" s="2">
         <v>5</v>
-      </c>
-      <c r="C4" s="2">
-        <v>400</v>
-      </c>
-      <c r="D4" s="2">
-        <v>4</v>
       </c>
       <c r="E4" s="2">
         <v>1</v>
@@ -992,13 +1072,13 @@
         <v>6</v>
       </c>
       <c r="C5" s="3">
-        <v>350</v>
+        <v>1500</v>
       </c>
       <c r="D5" s="3">
         <v>3</v>
       </c>
       <c r="E5" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1009,13 +1089,13 @@
         <v>6</v>
       </c>
       <c r="C6" s="2">
-        <v>450</v>
+        <v>0</v>
       </c>
       <c r="D6" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>